<commit_message>
Add ignore_errors option to xlrange
This commit adds a new boolean `ignore_errors` parameter to the `xlrange` table function, allowing callers to suppress parse failures while reading spreadsheet data. It also updates the bundled DuckDB binary and example workbook used for validation.
</commit_message>
<xml_diff>
--- a/examples/test_cases.xlsx
+++ b/examples/test_cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\src\examples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\DuckDBExcelAddin\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC94A30E-952F-4671-87DC-3F26E007904F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D22DBA-1C5D-435F-A5C9-8C8B74C7DC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{16A29E05-5294-4C93-91C1-6C3B8F27AE65}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{16A29E05-5294-4C93-91C1-6C3B8F27AE65}"/>
   </bookViews>
   <sheets>
     <sheet name="TYPES" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -66,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="113">
   <si>
     <t>select 1::tinyint</t>
   </si>
@@ -396,6 +393,18 @@
   </si>
   <si>
     <t>with integer</t>
+  </si>
+  <si>
+    <t>IGNORE_ERRORS=FALSE</t>
+  </si>
+  <si>
+    <t>select * from xlrange(1, strict=false, sample=2)</t>
+  </si>
+  <si>
+    <t>IGNORE_ERRORS=TRUE</t>
+  </si>
+  <si>
+    <t>select * from xlrange(1, strict=false, sample=2, ignore_errors=true)</t>
   </si>
 </sst>
 </file>
@@ -462,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -475,7 +484,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -796,16 +804,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5358680-0ED5-4EFA-AB03-B446D1F523DD}">
   <dimension ref="A1:B110"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="72.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.77734375" customWidth="1"/>
-    <col min="7" max="7" width="38.109375" customWidth="1"/>
+    <col min="2" max="2" width="72.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="38.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -813,18 +821,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="str" cm="1">
         <f t="array" ref="B2:B3">_xll.DUCKDB.EXEC(B1)</f>
         <v>CAST(1 AS "TINYINT")</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -832,18 +840,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="str" cm="1">
         <f t="array" ref="B6:B7">_xll.DUCKDB.EXEC(B5)</f>
         <v>CAST(1 AS "UTINYINT")</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -851,18 +859,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="str" cm="1">
         <f t="array" ref="B10:B11">_xll.DUCKDB.EXEC(B9)</f>
         <v>CAST(1 AS SMALLINT)</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -870,18 +878,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="str" cm="1">
         <f t="array" ref="B14:B15">_xll.DUCKDB.EXEC(B13)</f>
         <v>CAST(1 AS "USMALLINT")</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -889,18 +897,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="str" cm="1">
         <f t="array" ref="B18:B19">_xll.DUCKDB.EXEC(B17)</f>
         <v>CAST(1 AS INTEGER)</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B19" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -908,18 +916,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="str" cm="1">
         <f t="array" ref="B22:B23">_xll.DUCKDB.EXEC(B21)</f>
         <v>CAST(1 AS "UINTEGER")</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B23" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -927,18 +935,18 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="str" cm="1">
         <f t="array" ref="B26:B27">_xll.DUCKDB.EXEC(B25)</f>
         <v>CAST(1 AS BIGINT)</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B27" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -946,18 +954,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="str" cm="1">
         <f t="array" ref="B30:B31">_xll.DUCKDB.EXEC(B29)</f>
         <v>CAST(1 AS "UBIGINT")</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B31" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>24</v>
       </c>
@@ -965,18 +973,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B34" s="2" t="str" cm="1">
         <f t="array" ref="B34:B35">_xll.DUCKDB.EXEC(B33)</f>
         <v>CAST(1 AS "HUGEINT")</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B35" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>25</v>
       </c>
@@ -984,18 +992,18 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B38" s="2" t="str" cm="1">
         <f t="array" ref="B38:B39">_xll.DUCKDB.EXEC(B37)</f>
         <v>CAST(1 AS "UHUGEINT")</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1003,18 +1011,18 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="str" cm="1">
         <f t="array" ref="B42:B43">_xll.DUCKDB.EXEC(B41)</f>
         <v>CAST('t' AS BOOLEAN)</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -1022,18 +1030,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="str" cm="1">
         <f t="array" ref="B46:B47">_xll.DUCKDB.EXEC(B45)</f>
         <v>'abc'</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="str">
         <v>abc</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -1041,18 +1049,18 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="str" cm="1">
         <f t="array" ref="B50:B51">_xll.DUCKDB.EXEC(B49)</f>
         <v>CAST(1.2 AS FLOAT)</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B51" s="2">
         <v>1.2000000476837158</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>18</v>
       </c>
@@ -1060,18 +1068,18 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="str" cm="1">
         <f t="array" ref="B54:B55">_xll.DUCKDB.EXEC(B53)</f>
         <v>CAST(1.2 AS "DOUBLE")</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B55" s="2">
         <v>1.2</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>28</v>
       </c>
@@ -1079,18 +1087,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="str" cm="1">
         <f t="array" ref="B58:B59">_xll.DUCKDB.EXEC(B57)</f>
         <v>CAST(1.2 AS DECIMAL(4, 2))</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B59" s="2">
         <v>1.2</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>30</v>
       </c>
@@ -1098,18 +1106,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="str" cm="1">
         <f t="array" ref="B62:B63">_xll.DUCKDB.EXEC(B61)</f>
         <v>CAST(1.2 AS DECIMAL(9, 2))</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B63" s="2">
         <v>1.2</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>32</v>
       </c>
@@ -1117,18 +1125,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="str" cm="1">
         <f t="array" ref="B66:B67">_xll.DUCKDB.EXEC(B65)</f>
         <v>CAST(1.2 AS DECIMAL(18, 2))</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B67" s="2">
         <v>1.2</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>34</v>
       </c>
@@ -1136,18 +1144,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="str" cm="1">
         <f t="array" ref="B70:B71">_xll.DUCKDB.EXEC(B69)</f>
         <v>CAST(1.2 AS DECIMAL(38, 2))</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B71" s="2">
         <v>1.2</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>36</v>
       </c>
@@ -1155,18 +1163,18 @@
         <v>37</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="str" cm="1">
         <f t="array" ref="B74:B75">_xll.DUCKDB.EXEC(B73)</f>
         <v>CAST('2026-12-31' AS "DATE")</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B75" s="4">
         <v>46387</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>38</v>
       </c>
@@ -1174,18 +1182,18 @@
         <v>39</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="str" cm="1">
         <f t="array" ref="B78:B79">_xll.DUCKDB.EXEC(B77)</f>
         <v>CAST('09:30:45' AS TIME)</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B79" s="5">
         <v>0.39635416666666667</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>40</v>
       </c>
@@ -1193,18 +1201,18 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="str" cm="1">
         <f t="array" ref="B82:B83">_xll.DUCKDB.EXEC(B81)</f>
         <v>CAST('09:30:45+07:00' AS "TIME WITH TIME ZONE")</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B83" s="5">
         <v>0.39635416666666667</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>42</v>
       </c>
@@ -1212,18 +1220,18 @@
         <v>43</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="str" cm="1">
         <f t="array" ref="B86:B87">_xll.DUCKDB.EXEC(B85)</f>
         <v>CAST('2026-12-31 09:30:45' AS TIMESTAMP)</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B87" s="6">
         <v>46387.396354166667</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>44</v>
       </c>
@@ -1231,18 +1239,18 @@
         <v>45</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="str" cm="1">
         <f t="array" ref="B90:B91">_xll.DUCKDB.EXEC(B89)</f>
         <v>CAST('2026-12-31 09:30:45+07:00' AS "TIMESTAMP WITH TIME ZONE")</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B91" s="6">
         <v>46387.104687500003</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>46</v>
       </c>
@@ -1250,18 +1258,18 @@
         <v>47</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="str" cm="1">
         <f t="array" ref="B94:B95">_xll.DUCKDB.EXEC(B93)</f>
         <v>CAST('2026-12-31 09:30:45' AS "TIMESTAMP_S")</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B95" s="6">
         <v>46387.396354166667</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>48</v>
       </c>
@@ -1269,18 +1277,18 @@
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="str" cm="1">
         <f t="array" ref="B98:B99">_xll.DUCKDB.EXEC(B97)</f>
         <v>CAST('2026-12-31 09:30:45' AS "TIMESTAMP_MS")</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B99" s="6">
         <v>46387.396354166667</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>50</v>
       </c>
@@ -1288,18 +1296,18 @@
         <v>51</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="str" cm="1">
         <f t="array" ref="B102:B103">_xll.DUCKDB.EXEC(B101)</f>
         <v>CAST('2026-12-31 09:30:45' AS "TIMESTAMP_NS")</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B103" s="6">
         <v>46387.396354166667</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>52</v>
       </c>
@@ -1307,18 +1315,18 @@
         <v>53</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="str" cm="1">
         <f t="array" ref="B106:B107">_xll.DUCKDB.EXEC(B105)</f>
         <v>NULL</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>54</v>
       </c>
@@ -1326,10 +1334,10 @@
         <v>83</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="str" cm="1">
         <f t="array" ref="B110">_xll.DUCKDB.EXEC(B109)</f>
-        <v>Error fetching data: Column my_column: Unsupported DuckDB type. Convert the value to VARCHAR before returning it to Excel</v>
+        <v>Error fetching data: Column my_column: Unsupported DuckDB type. Convert the value to VARCHAR before returning it to Excel.</v>
       </c>
     </row>
   </sheetData>
@@ -1340,18 +1348,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751A3194-2367-4BAA-BC32-C926CD8293A5}">
-  <dimension ref="A1:G97"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G106"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.77734375" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" customWidth="1"/>
-    <col min="5" max="5" width="14.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="1" max="1" width="48.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>91</v>
       </c>
@@ -1371,7 +1379,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>1</v>
       </c>
@@ -1386,7 +1394,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1.2</v>
       </c>
@@ -1397,7 +1405,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1.3</v>
       </c>
@@ -1408,7 +1416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -1416,7 +1424,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7" t="str" cm="1">
         <f t="array" ref="B7:F8">_xll.DUCKDB.EXEC(B6,$B$1:$F$2)</f>
         <v>NUMBER_1</v>
@@ -1434,7 +1442,7 @@
         <v>ERROR_COL</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>1</v>
       </c>
@@ -1451,12 +1459,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" t="str" cm="1">
         <f t="array" ref="B11:G16">_xll.DUCKDB.EXEC(B10,$B$1:$F$2)</f>
         <v>column_name</v>
@@ -1477,7 +1485,7 @@
         <v>extra</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <v>NUMBER_1</v>
       </c>
@@ -1497,7 +1505,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <v>NUMBER_2</v>
       </c>
@@ -1517,7 +1525,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <v>STRING_COL</v>
       </c>
@@ -1537,7 +1545,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <v>EMPTY_COL</v>
       </c>
@@ -1557,7 +1565,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <v>ERROR_COL</v>
       </c>
@@ -1577,7 +1585,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>64</v>
       </c>
@@ -1585,7 +1593,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B19" t="str" cm="1">
         <f t="array" ref="B19:F21">_xll.DUCKDB.EXEC(B18,$B$1:$F$3)</f>
         <v>NUMBER_1</v>
@@ -1603,7 +1611,7 @@
         <v>ERROR_COL</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>1</v>
       </c>
@@ -1620,7 +1628,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>1.2</v>
       </c>
@@ -1637,12 +1645,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B24" t="str" cm="1">
         <f t="array" ref="B24:G29">_xll.DUCKDB.EXEC(B23,$B$1:$F$3)</f>
         <v>column_name</v>
@@ -1663,7 +1671,7 @@
         <v>extra</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>65</v>
       </c>
@@ -1686,7 +1694,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <v>NUMBER_2</v>
       </c>
@@ -1706,7 +1714,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
         <v>STRING_COL</v>
       </c>
@@ -1726,7 +1734,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
         <v>EMPTY_COL</v>
       </c>
@@ -1746,7 +1754,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
         <v>ERROR_COL</v>
       </c>
@@ -1766,7 +1774,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>67</v>
       </c>
@@ -1774,7 +1782,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B32" t="str" cm="1">
         <f t="array" ref="B32:F35">_xll.DUCKDB.EXEC(B31,$B$1:$F$4)</f>
         <v>NUMBER_1</v>
@@ -1792,7 +1800,7 @@
         <v>ERROR_COL</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B33">
         <v>1</v>
       </c>
@@ -1809,7 +1817,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B34">
         <v>1.2</v>
       </c>
@@ -1826,7 +1834,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B35">
         <v>1.3</v>
       </c>
@@ -1843,12 +1851,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B37" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B38" t="str" cm="1">
         <f t="array" ref="B38:G43">_xll.DUCKDB.EXEC(B37,$B$1:$F$4)</f>
         <v>column_name</v>
@@ -1869,7 +1877,7 @@
         <v>extra</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" t="str">
         <v>NUMBER_1</v>
@@ -1890,7 +1898,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>66</v>
       </c>
@@ -1913,7 +1921,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B41" t="str">
         <v>STRING_COL</v>
       </c>
@@ -1933,7 +1941,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B42" t="str">
         <v>EMPTY_COL</v>
       </c>
@@ -1953,7 +1961,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="str">
         <v>ERROR_COL</v>
       </c>
@@ -1973,7 +1981,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>68</v>
       </c>
@@ -1981,13 +1989,13 @@
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B46" t="str" cm="1">
         <f t="array" ref="B46">_xll.DUCKDB.EXEC(B45,$B$1:$F$4)</f>
-        <v>Invalid Input Error: Error scanning xlrange: Column NUMBER_1, row 3: Failed to convert to INTEGER</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Invalid Input Error: Error scanning xlrange: Column NUMBER_1, row 3: Failed to convert value to INTEGER.</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>69</v>
       </c>
@@ -1995,7 +2003,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B49" t="str" cm="1">
         <f t="array" ref="B49:G54">_xll.DUCKDB.EXEC(B48,$B$1:$F$4)</f>
         <v>column_name</v>
@@ -2016,7 +2024,7 @@
         <v>extra</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B50" t="str">
         <v>NUMBER_1</v>
       </c>
@@ -2036,7 +2044,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B51" t="str">
         <v>NUMBER_2</v>
       </c>
@@ -2056,7 +2064,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B52" t="str">
         <v>STRING_COL</v>
       </c>
@@ -2076,7 +2084,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B53" t="str">
         <v>EMPTY_COL</v>
       </c>
@@ -2096,7 +2104,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B54" t="str">
         <v>ERROR_COL</v>
       </c>
@@ -2116,7 +2124,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>71</v>
       </c>
@@ -2124,7 +2132,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B57" t="str" cm="1">
         <f t="array" ref="B57:G62">_xll.DUCKDB.EXEC(B56,$B$1:$F$4)</f>
         <v>column_name</v>
@@ -2145,7 +2153,7 @@
         <v>extra</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B58" t="str">
         <v>NUMBER_1</v>
       </c>
@@ -2165,7 +2173,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B59" t="str">
         <v>NUMBER_2</v>
       </c>
@@ -2185,7 +2193,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B60" t="str">
         <v>STRING_COL</v>
       </c>
@@ -2205,7 +2213,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B61" t="str">
         <v>EMPTY_COL</v>
       </c>
@@ -2225,7 +2233,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B62" t="str">
         <v>ERROR_COL</v>
       </c>
@@ -2245,7 +2253,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>89</v>
       </c>
@@ -2253,7 +2261,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B65" t="str" cm="1">
         <f t="array" ref="B65:F69">_xll.DUCKDB.EXEC(B64,B1:F4)</f>
         <v>column_0</v>
@@ -2271,7 +2279,7 @@
         <v>column_4</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B66" t="str">
         <v>NUMBER_1</v>
       </c>
@@ -2288,7 +2296,7 @@
         <v>ERROR_COL</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B67" t="str">
         <v>1</v>
       </c>
@@ -2305,7 +2313,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B68" t="str">
         <v>1.2</v>
       </c>
@@ -2322,7 +2330,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B69" t="str">
         <v>1.3</v>
       </c>
@@ -2339,7 +2347,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>92</v>
       </c>
@@ -2350,7 +2358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B72">
         <v>1</v>
       </c>
@@ -2364,7 +2372,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B73">
         <v>1.2</v>
       </c>
@@ -2375,7 +2383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B74">
         <v>1.3</v>
       </c>
@@ -2389,7 +2397,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>94</v>
       </c>
@@ -2397,7 +2405,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B77" t="str" cm="1">
         <f t="array" ref="B77">_xll.DUCKDB.EXEC(B76,B71:E74)</f>
         <v>Binder Error: Error binding xlrange: Column #2: Invalid column name. Column names must be non-empty and valid DuckDB identifiers.
@@ -2405,7 +2413,7 @@
                       ^</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>96</v>
       </c>
@@ -2413,7 +2421,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B80" t="str" cm="1">
         <f t="array" ref="B80:E83">_xll.DUCKDB.EXEC(B79,B71:E74)</f>
         <v>col1</v>
@@ -2428,7 +2436,7 @@
         <v>unnamed_1</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B81">
         <v>1</v>
       </c>
@@ -2442,7 +2450,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B82">
         <v>1.2</v>
       </c>
@@ -2456,7 +2464,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B83">
         <v>1.3</v>
       </c>
@@ -2470,7 +2478,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>98</v>
       </c>
@@ -2481,7 +2489,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B86">
         <v>1</v>
       </c>
@@ -2489,7 +2497,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B87">
         <v>1.2</v>
       </c>
@@ -2497,7 +2505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B88">
         <v>1.3</v>
       </c>
@@ -2506,7 +2514,7 @@
       </c>
       <c r="E88" s="9"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>94</v>
       </c>
@@ -2514,7 +2522,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B91" t="str" cm="1">
         <f t="array" ref="B91">_xll.DUCKDB.EXEC(B90,B85:C88)</f>
         <v>Binder Error: table "xlrange" has duplicate column name "dup"
@@ -2522,7 +2530,7 @@
                       ^</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>96</v>
       </c>
@@ -2530,7 +2538,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B94" t="str" cm="1">
         <f t="array" ref="B94:C97">_xll.DUCKDB.EXEC(B93,B85:C88)</f>
         <v>dup</v>
@@ -2539,7 +2547,7 @@
         <v>dup_1</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B95">
         <v>1</v>
       </c>
@@ -2547,7 +2555,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B96">
         <v>1.2</v>
       </c>
@@ -2555,12 +2563,67 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <v>1.3</v>
       </c>
       <c r="C97" t="str">
         <v>abc</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>109</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B100" t="str" cm="1">
+        <f t="array" ref="B100">_xll.DUCKDB.EXEC(B99,B85:C88)</f>
+        <v>Invalid Input Error: Error scanning xlrange: Column dup_1, row 4: Failed to convert value to DOUBLE.</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>111</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B103" t="str" cm="1">
+        <f t="array" ref="B103:C106">_xll.DUCKDB.EXEC(B102,B85:C88)</f>
+        <v>dup</v>
+      </c>
+      <c r="C103" t="str">
+        <v>dup_1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B104">
+        <v>1</v>
+      </c>
+      <c r="C104">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B105">
+        <v>1.2</v>
+      </c>
+      <c r="C105">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B106">
+        <v>1.3</v>
+      </c>
+      <c r="C106" t="e">
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>
@@ -2571,17 +2634,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A836AEC-DD0A-4797-B454-6E20C81CB53A}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" customWidth="1"/>
-    <col min="4" max="4" width="24.109375" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -2595,18 +2658,18 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="9">
         <v>46387</v>
       </c>
-      <c r="C2" s="11">
+      <c r="C2" s="10">
         <v>0.39635416666666667</v>
       </c>
       <c r="D2" s="6">
         <v>46387.396354166667</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>104</v>
       </c>
@@ -2614,7 +2677,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>105</v>
       </c>
@@ -2629,21 +2692,18 @@
         <v>CAST(xldatetime(CAST(datetime_col AS "DOUBLE")) AS VARCHAR)</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="str">
         <v>2026-12-31</v>
       </c>
-      <c r="C6" s="12" t="str">
+      <c r="C6" s="11" t="str">
         <v>09:30:45</v>
       </c>
       <c r="D6" s="6" t="str">
         <v>2026-12-31 09:30:45</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G7" s="10"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>104</v>
       </c>
@@ -2651,7 +2711,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>108</v>
       </c>
@@ -2666,7 +2726,7 @@
         <v>CAST(xldatetime(CAST(datetime_col AS INTEGER)) AS VARCHAR)</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="str">
         <v>2026-12-31</v>
       </c>
@@ -2685,13 +2745,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66184BE2-F564-4E42-8CE8-BFC8C65E358F}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>86</v>
       </c>
@@ -2699,23 +2759,23 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" t="str" cm="1">
         <f t="array" ref="B3:B4">_xll.DUCKDB.EXECX(B1,B2)</f>
         <v>test_macro(1)</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>100</v>
       </c>
@@ -2723,18 +2783,18 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="str" cm="1">
         <f t="array" ref="B7:B8">_xll.DUCKDB.EXECA(,B6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>103</v>
       </c>
@@ -2742,18 +2802,18 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="str" cm="1">
         <f t="array" ref="B12:B13">_xll.DUCKDB.EXECAX(,B10,B11)</f>
         <v>test_macro(1)</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>1</v>
       </c>
@@ -2766,13 +2826,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D42E5724-67A3-4259-906B-37F92D367239}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>73</v>
       </c>
@@ -2780,23 +2840,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" t="str" cm="1">
         <f t="array" ref="B3:B4">_xll.DUCKDB.EXEC(B2,B1)</f>
         <v>$1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -2804,23 +2864,23 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="str" cm="1">
         <f t="array" ref="B8:B9">_xll.DUCKDB.EXEC(B7,B6)</f>
         <v>$1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>1.2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -2828,23 +2888,23 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="str" cm="1">
         <f t="array" ref="B12:B13">_xll.DUCKDB.EXEC(B11,B10)</f>
         <v>$1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <v>abc</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2852,44 +2912,44 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B17" t="str" cm="1">
         <f t="array" ref="B17:B18">_xll.DUCKDB.EXEC(B16,B15)</f>
         <v>$1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B18" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B21" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B22" t="str" cm="1">
         <f t="array" ref="B22:B23">_xll.DUCKDB.EXEC(B21,B20)</f>
         <v>$1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B23" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>82</v>
       </c>
@@ -2898,15 +2958,15 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B26" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B27" t="str" cm="1">
         <f t="array" ref="B27">_xll.DUCKDB.EXEC(B26,B25)</f>
-        <v>Error: Parameter binding failed</v>
+        <v>Error: Parameter binding failed.</v>
       </c>
     </row>
   </sheetData>
@@ -2917,15 +2977,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C8C1CB2-5A89-4EE9-B7B8-26D912A856F1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="str" cm="1">
         <f t="array" ref="A1">_xll.DUCKDB.INFO()</f>
-        <v>Add-in version: v0.5.0
+        <v>Add-in version: v1.5.0
 DuckDB version: v1.5.5</v>
       </c>
     </row>
@@ -2937,17 +2997,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DE0166A-6705-4BE6-BC5D-3DDB4234D0EA}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -2956,12 +3016,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -2970,12 +3030,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>101</v>
       </c>
@@ -2984,12 +3044,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>102</v>
       </c>
@@ -2998,7 +3058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>1</v>
       </c>
@@ -3011,23 +3071,23 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65879F08-AA5E-452D-9515-58424370F18B}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" customWidth="1"/>
+    <col min="1" max="1" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
         <f t="array" ref="A2:A3">_xll.DUCKDB.EXEC(A1)</f>
         <v>count_star()</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10</v>
       </c>

</xml_diff>